<commit_message>
Fix invisible cell borders (transparent alpha bug) and increase row height so wrapped text doesn't overflow
</commit_message>
<xml_diff>
--- a/Jeopardy Answer Form.xlsx
+++ b/Jeopardy Answer Form.xlsx
@@ -90,16 +90,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00B7BFD1"/>
+        <color rgb="FF6B7590"/>
       </left>
       <right style="thin">
-        <color rgb="00B7BFD1"/>
+        <color rgb="FF6B7590"/>
       </right>
       <top style="thin">
-        <color rgb="00B7BFD1"/>
+        <color rgb="FF6B7590"/>
       </top>
       <bottom style="thin">
-        <color rgb="00B7BFD1"/>
+        <color rgb="FF6B7590"/>
       </bottom>
     </border>
   </borders>
@@ -582,7 +582,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
+    <row r="2" ht="60" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Firsts &amp; Milestones</t>
@@ -598,7 +598,7 @@
       </c>
       <c r="D2" s="7" t="inlineStr"/>
     </row>
-    <row r="3" ht="30" customHeight="1">
+    <row r="3" ht="60" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Firsts &amp; Milestones</t>
@@ -614,7 +614,7 @@
       </c>
       <c r="D3" s="7" t="inlineStr"/>
     </row>
-    <row r="4" ht="30" customHeight="1">
+    <row r="4" ht="60" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Firsts &amp; Milestones</t>
@@ -630,7 +630,7 @@
       </c>
       <c r="D4" s="7" t="inlineStr"/>
     </row>
-    <row r="5" ht="30" customHeight="1">
+    <row r="5" ht="60" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Firsts &amp; Milestones</t>
@@ -646,7 +646,7 @@
       </c>
       <c r="D5" s="7" t="inlineStr"/>
     </row>
-    <row r="6" ht="30" customHeight="1">
+    <row r="6" ht="60" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Firsts &amp; Milestones</t>
@@ -658,7 +658,7 @@
       <c r="C6" s="5" t="inlineStr"/>
       <c r="D6" s="7" t="inlineStr"/>
     </row>
-    <row r="7" ht="30" customHeight="1">
+    <row r="7" ht="60" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
           <t>All About Your Fiancé</t>
@@ -674,7 +674,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr"/>
     </row>
-    <row r="8" ht="30" customHeight="1">
+    <row r="8" ht="60" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
           <t>All About Your Fiancé</t>
@@ -690,7 +690,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr"/>
     </row>
-    <row r="9" ht="30" customHeight="1">
+    <row r="9" ht="60" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
           <t>All About Your Fiancé</t>
@@ -706,7 +706,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr"/>
     </row>
-    <row r="10" ht="30" customHeight="1">
+    <row r="10" ht="60" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
           <t>All About Your Fiancé</t>
@@ -722,7 +722,7 @@
       </c>
       <c r="D10" s="7" t="inlineStr"/>
     </row>
-    <row r="11" ht="30" customHeight="1">
+    <row r="11" ht="60" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
           <t>All About Your Fiancé</t>
@@ -738,7 +738,7 @@
       </c>
       <c r="D11" s="7" t="inlineStr"/>
     </row>
-    <row r="12" ht="30" customHeight="1">
+    <row r="12" ht="60" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
           <t>All About You</t>
@@ -754,7 +754,7 @@
       </c>
       <c r="D12" s="7" t="inlineStr"/>
     </row>
-    <row r="13" ht="30" customHeight="1">
+    <row r="13" ht="60" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
           <t>All About You</t>
@@ -770,7 +770,7 @@
       </c>
       <c r="D13" s="7" t="inlineStr"/>
     </row>
-    <row r="14" ht="30" customHeight="1">
+    <row r="14" ht="60" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
           <t>All About You</t>
@@ -786,7 +786,7 @@
       </c>
       <c r="D14" s="7" t="inlineStr"/>
     </row>
-    <row r="15" ht="30" customHeight="1">
+    <row r="15" ht="60" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
           <t>All About You</t>
@@ -802,7 +802,7 @@
       </c>
       <c r="D15" s="7" t="inlineStr"/>
     </row>
-    <row r="16" ht="30" customHeight="1">
+    <row r="16" ht="60" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
           <t>All About You</t>
@@ -814,7 +814,7 @@
       <c r="C16" s="5" t="inlineStr"/>
       <c r="D16" s="7" t="inlineStr"/>
     </row>
-    <row r="17" ht="30" customHeight="1">
+    <row r="17" ht="60" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Pet Peeves &amp; Habits</t>
@@ -830,7 +830,7 @@
       </c>
       <c r="D17" s="7" t="inlineStr"/>
     </row>
-    <row r="18" ht="30" customHeight="1">
+    <row r="18" ht="60" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Pet Peeves &amp; Habits</t>
@@ -846,7 +846,7 @@
       </c>
       <c r="D18" s="7" t="inlineStr"/>
     </row>
-    <row r="19" ht="30" customHeight="1">
+    <row r="19" ht="60" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Pet Peeves &amp; Habits</t>
@@ -862,7 +862,7 @@
       </c>
       <c r="D19" s="7" t="inlineStr"/>
     </row>
-    <row r="20" ht="30" customHeight="1">
+    <row r="20" ht="60" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
           <t>Pet Peeves &amp; Habits</t>
@@ -878,7 +878,7 @@
       </c>
       <c r="D20" s="7" t="inlineStr"/>
     </row>
-    <row r="21" ht="30" customHeight="1">
+    <row r="21" ht="60" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Pet Peeves &amp; Habits</t>
@@ -890,7 +890,7 @@
       <c r="C21" s="5" t="inlineStr"/>
       <c r="D21" s="7" t="inlineStr"/>
     </row>
-    <row r="22" ht="30" customHeight="1">
+    <row r="22" ht="60" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Shared Memories</t>
@@ -906,7 +906,7 @@
       </c>
       <c r="D22" s="7" t="inlineStr"/>
     </row>
-    <row r="23" ht="30" customHeight="1">
+    <row r="23" ht="60" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Shared Memories</t>
@@ -922,7 +922,7 @@
       </c>
       <c r="D23" s="7" t="inlineStr"/>
     </row>
-    <row r="24" ht="30" customHeight="1">
+    <row r="24" ht="60" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
           <t>Shared Memories</t>
@@ -934,7 +934,7 @@
       <c r="C24" s="5" t="inlineStr"/>
       <c r="D24" s="7" t="inlineStr"/>
     </row>
-    <row r="25" ht="30" customHeight="1">
+    <row r="25" ht="60" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
           <t>Shared Memories</t>
@@ -946,7 +946,7 @@
       <c r="C25" s="5" t="inlineStr"/>
       <c r="D25" s="7" t="inlineStr"/>
     </row>
-    <row r="26" ht="30" customHeight="1">
+    <row r="26" ht="60" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
         <is>
           <t>Shared Memories</t>

</xml_diff>